<commit_message>
fix(retrain): drop null-hit rows + 100%-null cols in build_retrain_dataset
- Added null-hit row filter (51K clean rows vs 124K with 59% null hit)
- Added 99%-null column drop (36 cols removed)
- TRAINING_FROM_DATE default stays 2026-05-06 (Soccer opp fix boundary)
- --from '' override works for full history when needed

New production model: 0.7673 overall (all per-sport gates pass)
  MLB 0.7344, NBA 0.6025, NHL 0.7732, Soccer 0.5551, WNBA 0.7032
Previous backup: pre_retrain_2026-05-21 (0.7743 on 395K rows, not reproducible)
Step8 files exist 2026-03-01 to 2026-05-27 (87 dates)

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-25.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-25.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="E2" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F2" t="n">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="G2" t="n">
-        <v>67.8</v>
+        <v>56.8</v>
       </c>
     </row>
     <row r="3">
@@ -500,16 +500,16 @@
         </is>
       </c>
       <c r="D3" t="n">
+        <v>83</v>
+      </c>
+      <c r="E3" t="n">
+        <v>44</v>
+      </c>
+      <c r="F3" t="n">
+        <v>39</v>
+      </c>
+      <c r="G3" t="n">
         <v>53</v>
-      </c>
-      <c r="E3" t="n">
-        <v>32</v>
-      </c>
-      <c r="F3" t="n">
-        <v>21</v>
-      </c>
-      <c r="G3" t="n">
-        <v>60.4</v>
       </c>
     </row>
     <row r="4">
@@ -529,16 +529,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>60</v>
+        <v>135</v>
       </c>
       <c r="E4" t="n">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="F4" t="n">
-        <v>34</v>
+        <v>77</v>
       </c>
       <c r="G4" t="n">
-        <v>43.3</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5">
@@ -558,16 +558,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E5" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F5" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G5" t="n">
-        <v>64.40000000000001</v>
+        <v>58.1</v>
       </c>
     </row>
     <row r="6">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="E6" t="n">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="F6" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="G6" t="n">
-        <v>46.2</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="E7" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="F7" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G7" t="n">
-        <v>61.4</v>
+        <v>61.8</v>
       </c>
     </row>
     <row r="8">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>470</v>
+        <v>413</v>
       </c>
       <c r="E8" t="n">
-        <v>145</v>
+        <v>124</v>
       </c>
       <c r="F8" t="n">
-        <v>325</v>
+        <v>289</v>
       </c>
       <c r="G8" t="n">
-        <v>30.9</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="E9" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="F9" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="G9" t="n">
-        <v>59.7</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>478</v>
+        <v>198</v>
       </c>
       <c r="E10" t="n">
-        <v>280</v>
+        <v>130</v>
       </c>
       <c r="F10" t="n">
-        <v>198</v>
+        <v>68</v>
       </c>
       <c r="G10" t="n">
-        <v>58.6</v>
+        <v>65.7</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>277</v>
+        <v>851</v>
       </c>
       <c r="E11" t="n">
-        <v>159</v>
+        <v>516</v>
       </c>
       <c r="F11" t="n">
-        <v>118</v>
+        <v>335</v>
       </c>
       <c r="G11" t="n">
-        <v>57.4</v>
+        <v>60.6</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E12" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F12" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G12" t="n">
-        <v>57.2</v>
+        <v>58.2</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="E13" t="n">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="F13" t="n">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="G13" t="n">
-        <v>41.9</v>
+        <v>42.4</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="E14" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F14" t="n">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="G14" t="n">
-        <v>18.4</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>126</v>
+        <v>194</v>
       </c>
       <c r="E15" t="n">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="F15" t="n">
-        <v>105</v>
+        <v>160</v>
       </c>
       <c r="G15" t="n">
-        <v>16.7</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="16">
@@ -877,16 +877,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="E16" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F16" t="n">
-        <v>63</v>
+        <v>80</v>
       </c>
       <c r="G16" t="n">
-        <v>18.2</v>
+        <v>19.2</v>
       </c>
     </row>
     <row r="17">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2960</v>
+        <v>3260</v>
       </c>
       <c r="E17" t="n">
-        <v>500</v>
+        <v>670</v>
       </c>
       <c r="F17" t="n">
-        <v>2460</v>
+        <v>2590</v>
       </c>
       <c r="G17" t="n">
-        <v>16.9</v>
+        <v>20.6</v>
       </c>
     </row>
   </sheetData>
@@ -1172,7 +1172,7 @@
         <v>10</v>
       </c>
       <c r="X2" t="n">
-        <v>17</v>
+        <v>17.6</v>
       </c>
       <c r="Y2" t="n">
         <v>188</v>
@@ -1471,100 +1471,100 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>58.6</v>
+        <v>65.7</v>
       </c>
       <c r="C7" t="n">
-        <v>478</v>
+        <v>198</v>
       </c>
       <c r="D7" t="n">
-        <v>57.4</v>
+        <v>60.6</v>
       </c>
       <c r="E7" t="n">
-        <v>277</v>
+        <v>851</v>
       </c>
       <c r="F7" t="n">
-        <v>57.2</v>
+        <v>58.2</v>
       </c>
       <c r="G7" t="n">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="H7" t="n">
-        <v>41.9</v>
+        <v>42.4</v>
       </c>
       <c r="I7" t="n">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="J7" t="n">
-        <v>18.4</v>
+        <v>17.6</v>
       </c>
       <c r="K7" t="n">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="L7" t="n">
-        <v>16.7</v>
+        <v>17.5</v>
       </c>
       <c r="M7" t="n">
-        <v>126</v>
+        <v>194</v>
       </c>
       <c r="N7" t="n">
-        <v>18.2</v>
+        <v>19.2</v>
       </c>
       <c r="O7" t="n">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="P7" t="n">
-        <v>16.9</v>
+        <v>20.6</v>
       </c>
       <c r="Q7" t="n">
-        <v>2960</v>
+        <v>3260</v>
       </c>
       <c r="R7" t="n">
-        <v>67.8</v>
+        <v>56.8</v>
       </c>
       <c r="S7" t="n">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="T7" t="n">
-        <v>43.3</v>
+        <v>43</v>
       </c>
       <c r="U7" t="n">
+        <v>135</v>
+      </c>
+      <c r="V7" t="n">
+        <v>31</v>
+      </c>
+      <c r="W7" t="n">
+        <v>29</v>
+      </c>
+      <c r="X7" t="n">
+        <v>30</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>413</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>53</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>83</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>58.1</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>43</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>34</v>
+      </c>
+      <c r="AF7" t="n">
         <v>60</v>
       </c>
-      <c r="V7" t="n">
-        <v>46.2</v>
-      </c>
-      <c r="W7" t="n">
-        <v>52</v>
-      </c>
-      <c r="X7" t="n">
-        <v>30.9</v>
-      </c>
-      <c r="Y7" t="n">
-        <v>470</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>60.4</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>53</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>64.40000000000001</v>
-      </c>
-      <c r="AC7" t="n">
-        <v>45</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>61.4</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>44</v>
-      </c>
-      <c r="AF7" t="n">
-        <v>59.7</v>
-      </c>
       <c r="AG7" t="n">
-        <v>176</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>